<commit_message>
Analysis-scope electrical report + string shunt diode + report CLI
- app.py: new 'report' CLI command; scope-driven from the analysis sheet (falls back to all phases)
- analysis sheet: schemas/analysis.py + loader/analysis.py; params.xlsx gains an 'analysis' sheet (single@EOL, dual@EOL) and a string_shunt_diode_reference_file row
- string shunt diode: ShuntDiodeParameters.v_forward + CellParameters.string_diode; loader reads both cell & string diodes; StringModel clamps the reverse-voltage tail; build_from_report threads it in
- data/diodes/aRoche.json: string shunt diode (placeholder)
- scripts/add_analysis_sheet.py: workbook patcher
- examples/build_noNG_elec_report.py: zero-install report wrapper
- Notes/: framework concept handbook (HTML) + figure script

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/params.xlsx
+++ b/params.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="structure" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mission_orbit" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mission_param" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="analysis" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -538,12 +539,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>diode_reference_file</t>
+          <t>cell_shunt_diode_reference_file</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Diode Reference File</t>
+          <t>Cell Shunt Diode's reference File</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -968,6 +969,28 @@
       <c r="F17" t="inlineStr">
         <is>
           <t>datasheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>string_shunt_diode_reference_file</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>String Shunt Diode's reference File</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>diodes/aRoche.json</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>path</t>
         </is>
       </c>
     </row>
@@ -3477,13 +3500,11 @@
           <t>Cell Parameters</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>cell_params</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>both</t>
@@ -3504,7 +3525,6 @@
           <t>Cell Radiation Regressors</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>figure</t>
@@ -3535,13 +3555,11 @@
           <t>Sections and Harness</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>sections_table</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>both</t>
@@ -3562,13 +3580,11 @@
           <t>Loss Factor Budget</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>loss_table</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>both</t>
@@ -3589,13 +3605,11 @@
           <t>Results</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>results_table</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>both</t>
@@ -3616,7 +3630,6 @@
           <t>Per-Section IV Curves by Wing and Position</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>figure</t>
@@ -3647,7 +3660,6 @@
           <t>Whole-Array IV/PV Curve</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>figure</t>
@@ -4913,4 +4925,113 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>launch</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>phase</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>season</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>temperature</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>string_loss</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>sun_angle</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>v_operating</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>End_of_Life</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1322/1367</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>101.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>dual</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>End_of_Life</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1322/1367</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>51.1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>101.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add mission requirement sheet + plot array output against it
- schemas/requirement.py + loader/requirement.py: load the 'requirement' sheet (operating voltage, EOR/EOL min power, max section current, sun angle, flux, magnetic moment)
- scripts/add_requirement_sheet.py: add the requirement sheet to a workbook
- app.py report: feed requirement into the report -- bus voltage falls back to voltage_operating; the P-V plot now draws the binding EOL/EOR minimum-power requirement line
- params.xlsx: requirement sheet added

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/params.xlsx
+++ b/params.xlsx
@@ -16,6 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mission_orbit" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mission_param" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="analysis" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="requirement" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -999,6 +1000,244 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>param</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>voltage_operating</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>101.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>voltage_unit</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>max_section_current</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>max_section_current_unit</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>magnetic_moment_max</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>magnetic_moment_unit</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Am^2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>eor_power_min</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>8350</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>eol_power_min</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>7550</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>power_unit</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>sun_angle</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>sun_angle_unit</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>deg</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>flux_at_array</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1321</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>flux_unit</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>W/m^2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add mission_orbit setter script; align bus_voltage + add max_beta_angle_deg
- scripts/set_mission_orbit.py: idempotent key-value setter for the mission_orbit sheet
- params.xlsx: bus_voltage 100 -> 101.5 V (matches requirement); add max_beta_angle_deg = 23.5 deg

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/params.xlsx
+++ b/params.xlsx
@@ -3926,7 +3926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4275,7 +4275,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>100</v>
+        <v>101.5</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -4308,6 +4308,31 @@
         </is>
       </c>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>max_beta_angle_deg</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Max Beta Angle</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>deg</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>float</t>
         </is>

</xml_diff>

<commit_message>
feat: reference the free-form circuit from params.xlsx; report runs from it
cell_params gains circuit_reference_file -> circuits/msro_nominal.json; build_params.py regenerated to include the row. Report now builds the array from the circuit (verified: single@EOL, dual@EOL).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/params.xlsx
+++ b/params.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -990,6 +990,28 @@
         </is>
       </c>
       <c r="E18" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>circuit_reference_file</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Circuit reference File</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>circuits/msro_nominal.json</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>path</t>
         </is>

</xml_diff>

<commit_message>
refactor(orbit): make view_factor_to_planet body_radius_km keyword-only; add guard test
</commit_message>
<xml_diff>
--- a/params.xlsx
+++ b/params.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -990,28 +990,6 @@
         </is>
       </c>
       <c r="E18" t="inlineStr">
-        <is>
-          <t>path</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>circuit_reference_file</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Circuit reference File</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>circuits/msro_nominal.json</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
         <is>
           <t>path</t>
         </is>

</xml_diff>

<commit_message>
feat(params): add bond_albedo/planet_temp_k/ir_emissivity to mission_orbit
</commit_message>
<xml_diff>
--- a/params.xlsx
+++ b/params.xlsx
@@ -3926,7 +3926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4333,6 +4333,81 @@
         </is>
       </c>
       <c r="E16" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>bond_albedo</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Bond Albedo</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>planet_temp_k</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Planet Temperature</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>255</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ir_emissivity</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Planet IR Emissivity</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>float</t>
         </is>

</xml_diff>

<commit_message>
feat: environmental power budget in thermal & Monte-Carlo reports
Add a per-m^2 power budget (incident solar, electrical extracted at the
~30% space-grade cell efficiency, albedo, planetary IR) with a worked
"show the calculation" block, to both the thermal and Monte-Carlo reports.

- view_factor_to_planet(altitude): geometric Earth view factor (GEO ~0.023)
- MissionOrbit schema + loader; mission_orbit sheet now loaded into
  ReportMetadata; bond_albedo/planet_temp_k/ir_emissivity added to params.xlsx
  and build_params.py
- analysis/power_budget.py: compute_power_budget() (pure)
- albedo/IR fed into the actual solve_thermal/solve_panel calls (Approach B);
  p_sun unchanged
- budget section + calculation rendered in both report templates

13 power-budget tests; full suite green; both report PDFs render the section.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/params.xlsx
+++ b/params.xlsx
@@ -3926,7 +3926,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4333,6 +4333,81 @@
         </is>
       </c>
       <c r="E16" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>bond_albedo</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Bond Albedo</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>planet_temp_k</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Planet Temperature</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>255</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ir_emissivity</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Planet IR Emissivity</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>float</t>
         </is>

</xml_diff>

<commit_message>
feat: substrate_reference_file + grid 3x2x12 layout + electrical&thermal report script
- schemas/cell.py + loader/cell.py: new substrate_reference_file on the cell (panel substrate optics/c_cond for the thermal report)
- params.xlsx: cell_params gains substrate_reference_file -> substrates/msro_case2.json
- analysis/thermal_report.py + render/thermal_report.py: run_thermal_report/ThermalReport accept a prebuilt PanelLayout (layout=) so one grid drives both reports
- app.py: build_electrical_report gains grid_file= override (derive the array from a given grid without changing the workbook)
- data/layouts/grid_3x2x12.json: 3 blocks x 2 parallel x 12 series = 72 cells (string/block tags + substrate optics + circuit)
- examples/build_grid_reports.py: generates the grid and BOTH the electrical and LaTeX thermal reports from that single grid
- tests: substrate_reference_file presence

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/params.xlsx
+++ b/params.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -990,6 +990,28 @@
         </is>
       </c>
       <c r="E18" t="inlineStr">
+        <is>
+          <t>path</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>substrate_reference_file</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Substrate reference File</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>substrates/msro_case2.json</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>path</t>
         </is>

</xml_diff>

<commit_message>
fix(percell): use real cell area in per-cell thermal solve (was diverging); merge condition layers into params.xlsx (single workbook)
</commit_message>
<xml_diff>
--- a/params.xlsx
+++ b/params.xlsx
@@ -17,6 +17,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mission_param" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="analysis" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="requirement" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="layer_state" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="layer_shade" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="layer_life" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="layer_incidence" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1238,6 +1242,490 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AE3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Cell state: 'healthy' (default) or 'failed_open'. Blank = healthy.</t>
+        </is>
+      </c>
+      <c r="B1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E1" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1" t="n">
+        <v>5</v>
+      </c>
+      <c r="H1" t="n">
+        <v>6</v>
+      </c>
+      <c r="I1" t="n">
+        <v>7</v>
+      </c>
+      <c r="J1" t="n">
+        <v>8</v>
+      </c>
+      <c r="K1" t="n">
+        <v>9</v>
+      </c>
+      <c r="L1" t="n">
+        <v>10</v>
+      </c>
+      <c r="M1" t="n">
+        <v>11</v>
+      </c>
+      <c r="N1" t="n">
+        <v>12</v>
+      </c>
+      <c r="O1" t="n">
+        <v>13</v>
+      </c>
+      <c r="P1" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q1" t="n">
+        <v>15</v>
+      </c>
+      <c r="R1" t="n">
+        <v>16</v>
+      </c>
+      <c r="S1" t="n">
+        <v>17</v>
+      </c>
+      <c r="T1" t="n">
+        <v>18</v>
+      </c>
+      <c r="U1" t="n">
+        <v>19</v>
+      </c>
+      <c r="V1" t="n">
+        <v>20</v>
+      </c>
+      <c r="W1" t="n">
+        <v>21</v>
+      </c>
+      <c r="X1" t="n">
+        <v>22</v>
+      </c>
+      <c r="Y1" t="n">
+        <v>23</v>
+      </c>
+      <c r="Z1" t="n">
+        <v>24</v>
+      </c>
+      <c r="AA1" t="n">
+        <v>25</v>
+      </c>
+      <c r="AB1" t="n">
+        <v>26</v>
+      </c>
+      <c r="AC1" t="n">
+        <v>27</v>
+      </c>
+      <c r="AD1" t="n">
+        <v>28</v>
+      </c>
+      <c r="AE1" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AE3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Irradiance transmittance [0..1]. 1.0 = unshaded (default). Blank = 1.0.</t>
+        </is>
+      </c>
+      <c r="B1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E1" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1" t="n">
+        <v>5</v>
+      </c>
+      <c r="H1" t="n">
+        <v>6</v>
+      </c>
+      <c r="I1" t="n">
+        <v>7</v>
+      </c>
+      <c r="J1" t="n">
+        <v>8</v>
+      </c>
+      <c r="K1" t="n">
+        <v>9</v>
+      </c>
+      <c r="L1" t="n">
+        <v>10</v>
+      </c>
+      <c r="M1" t="n">
+        <v>11</v>
+      </c>
+      <c r="N1" t="n">
+        <v>12</v>
+      </c>
+      <c r="O1" t="n">
+        <v>13</v>
+      </c>
+      <c r="P1" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q1" t="n">
+        <v>15</v>
+      </c>
+      <c r="R1" t="n">
+        <v>16</v>
+      </c>
+      <c r="S1" t="n">
+        <v>17</v>
+      </c>
+      <c r="T1" t="n">
+        <v>18</v>
+      </c>
+      <c r="U1" t="n">
+        <v>19</v>
+      </c>
+      <c r="V1" t="n">
+        <v>20</v>
+      </c>
+      <c r="W1" t="n">
+        <v>21</v>
+      </c>
+      <c r="X1" t="n">
+        <v>22</v>
+      </c>
+      <c r="Y1" t="n">
+        <v>23</v>
+      </c>
+      <c r="Z1" t="n">
+        <v>24</v>
+      </c>
+      <c r="AA1" t="n">
+        <v>25</v>
+      </c>
+      <c r="AB1" t="n">
+        <v>26</v>
+      </c>
+      <c r="AC1" t="n">
+        <v>27</v>
+      </c>
+      <c r="AD1" t="n">
+        <v>28</v>
+      </c>
+      <c r="AE1" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AE3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Mechanical chipping current-derate [0..1]. 1.0 = full (default). Blank = 1.0.</t>
+        </is>
+      </c>
+      <c r="B1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E1" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1" t="n">
+        <v>5</v>
+      </c>
+      <c r="H1" t="n">
+        <v>6</v>
+      </c>
+      <c r="I1" t="n">
+        <v>7</v>
+      </c>
+      <c r="J1" t="n">
+        <v>8</v>
+      </c>
+      <c r="K1" t="n">
+        <v>9</v>
+      </c>
+      <c r="L1" t="n">
+        <v>10</v>
+      </c>
+      <c r="M1" t="n">
+        <v>11</v>
+      </c>
+      <c r="N1" t="n">
+        <v>12</v>
+      </c>
+      <c r="O1" t="n">
+        <v>13</v>
+      </c>
+      <c r="P1" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q1" t="n">
+        <v>15</v>
+      </c>
+      <c r="R1" t="n">
+        <v>16</v>
+      </c>
+      <c r="S1" t="n">
+        <v>17</v>
+      </c>
+      <c r="T1" t="n">
+        <v>18</v>
+      </c>
+      <c r="U1" t="n">
+        <v>19</v>
+      </c>
+      <c r="V1" t="n">
+        <v>20</v>
+      </c>
+      <c r="W1" t="n">
+        <v>21</v>
+      </c>
+      <c r="X1" t="n">
+        <v>22</v>
+      </c>
+      <c r="Y1" t="n">
+        <v>23</v>
+      </c>
+      <c r="Z1" t="n">
+        <v>24</v>
+      </c>
+      <c r="AA1" t="n">
+        <v>25</v>
+      </c>
+      <c r="AB1" t="n">
+        <v>26</v>
+      </c>
+      <c r="AC1" t="n">
+        <v>27</v>
+      </c>
+      <c r="AD1" t="n">
+        <v>28</v>
+      </c>
+      <c r="AE1" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AE3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Cosine factor for blanket-bow incidence [0..1]. 1.0 = normal (default). Blank = 1.0.</t>
+        </is>
+      </c>
+      <c r="B1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E1" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1" t="n">
+        <v>4</v>
+      </c>
+      <c r="G1" t="n">
+        <v>5</v>
+      </c>
+      <c r="H1" t="n">
+        <v>6</v>
+      </c>
+      <c r="I1" t="n">
+        <v>7</v>
+      </c>
+      <c r="J1" t="n">
+        <v>8</v>
+      </c>
+      <c r="K1" t="n">
+        <v>9</v>
+      </c>
+      <c r="L1" t="n">
+        <v>10</v>
+      </c>
+      <c r="M1" t="n">
+        <v>11</v>
+      </c>
+      <c r="N1" t="n">
+        <v>12</v>
+      </c>
+      <c r="O1" t="n">
+        <v>13</v>
+      </c>
+      <c r="P1" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q1" t="n">
+        <v>15</v>
+      </c>
+      <c r="R1" t="n">
+        <v>16</v>
+      </c>
+      <c r="S1" t="n">
+        <v>17</v>
+      </c>
+      <c r="T1" t="n">
+        <v>18</v>
+      </c>
+      <c r="U1" t="n">
+        <v>19</v>
+      </c>
+      <c r="V1" t="n">
+        <v>20</v>
+      </c>
+      <c r="W1" t="n">
+        <v>21</v>
+      </c>
+      <c r="X1" t="n">
+        <v>22</v>
+      </c>
+      <c r="Y1" t="n">
+        <v>23</v>
+      </c>
+      <c r="Z1" t="n">
+        <v>24</v>
+      </c>
+      <c r="AA1" t="n">
+        <v>25</v>
+      </c>
+      <c r="AB1" t="n">
+        <v>26</v>
+      </c>
+      <c r="AC1" t="n">
+        <v>27</v>
+      </c>
+      <c r="AD1" t="n">
+        <v>28</v>
+      </c>
+      <c r="AE1" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>